<commit_message>
columna agregada de monto iva
</commit_message>
<xml_diff>
--- a/Output/resultado.xlsx
+++ b/Output/resultado.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,6 +437,11 @@
           <t>Categoria</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>MontoIva</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -444,7 +449,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PAGO 1</t>
+          <t>pago 1</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -454,6 +459,9 @@
         <is>
           <t>ventas</t>
         </is>
+      </c>
+      <c r="E2" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -462,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PAGO 2</t>
+          <t>pago 2</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -472,6 +480,9 @@
         <is>
           <t>gastos</t>
         </is>
+      </c>
+      <c r="E3" t="n">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>